<commit_message>
sprint reviews update + py lib instructions
</commit_message>
<xml_diff>
--- a/MongoDB/Sprint reviews.xlsx
+++ b/MongoDB/Sprint reviews.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10661916_polimi_it/Documents/PoliMi/4° anno/Corsi/Systems and Methods for Big and Unstructured Data/Project SMBUD/SMBUD DB/Repository/SMBUD-project2022/MongoDB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B11717F3-0734-46BC-9BDD-6E3B78836DA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{B11717F3-0734-46BC-9BDD-6E3B78836DA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A037A4B3-7DD4-4385-998A-641CFE34D941}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="348" windowWidth="23256" windowHeight="12720" xr2:uid="{40B4DD2A-A988-466C-98BC-3488A5760252}"/>
+    <workbookView xWindow="768" yWindow="1224" windowWidth="17280" windowHeight="9072" xr2:uid="{40B4DD2A-A988-466C-98BC-3488A5760252}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sprint reviews" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
-  <si>
-    <t>Sprint reviews</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
   <si>
     <t>Francesco</t>
   </si>
@@ -62,7 +59,22 @@
     <t>Expected</t>
   </si>
   <si>
-    <t>Analysis &amp; scheduling</t>
+    <t>Analysis</t>
+  </si>
+  <si>
+    <t>document schema</t>
+  </si>
+  <si>
+    <t>Learning Json py lib</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Check correctness document schema</t>
+  </si>
+  <si>
+    <t>Analysis, document schema</t>
   </si>
 </sst>
 </file>
@@ -98,11 +110,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -418,71 +435,98 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16F4F56A-16B6-413A-BB29-48CDE10B3DC3}">
-  <dimension ref="B2:G10"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.77734375" customWidth="1"/>
-    <col min="6" max="6" width="18.88671875" customWidth="1"/>
-    <col min="7" max="7" width="17.6640625" customWidth="1"/>
+    <col min="1" max="1" width="12.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" style="1"/>
+    <col min="3" max="6" width="17.88671875" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="3">
+        <v>44874</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3">
+        <v>44875</v>
+      </c>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="F4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="2:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="F5" s="2">
-        <v>44874</v>
-      </c>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="D6" t="s">
+      <c r="D3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F6" t="s">
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="D7" t="s">
-        <v>2</v>
-      </c>
-      <c r="F7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="D8" t="s">
-        <v>3</v>
-      </c>
-      <c r="F8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="D9" t="s">
+      <c r="D6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="D10" t="s">
-        <v>5</v>
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="F5:G5"/>
+  <mergeCells count="2">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Text extractor py completed + Sprint review update
</commit_message>
<xml_diff>
--- a/MongoDB/Sprint reviews.xlsx
+++ b/MongoDB/Sprint reviews.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10661916_polimi_it/Documents/PoliMi/4° anno/Corsi/Systems and Methods for Big and Unstructured Data/Project SMBUD/SMBUD DB/Repository/SMBUD-project2022/MongoDB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{B11717F3-0734-46BC-9BDD-6E3B78836DA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A037A4B3-7DD4-4385-998A-641CFE34D941}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="8_{B11717F3-0734-46BC-9BDD-6E3B78836DA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F27F2344-0197-4982-92EE-672E070AE912}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="1224" windowWidth="17280" windowHeight="9072" xr2:uid="{40B4DD2A-A988-466C-98BC-3488A5760252}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
   <si>
     <t>Francesco</t>
   </si>
@@ -75,14 +75,40 @@
   </si>
   <si>
     <t>Analysis, document schema</t>
+  </si>
+  <si>
+    <t>Latex template</t>
+  </si>
+  <si>
+    <t>Random data generation process</t>
+  </si>
+  <si>
+    <t>progress in random data generation</t>
+  </si>
+  <si>
+    <t>py from txt to json for book text</t>
+  </si>
+  <si>
+    <t>Learning about importing in MongoDB</t>
+  </si>
+  <si>
+    <t>?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -98,7 +124,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -106,20 +132,106 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -435,99 +547,152 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16F4F56A-16B6-413A-BB29-48CDE10B3DC3}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.88671875" style="1"/>
-    <col min="3" max="6" width="17.88671875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="5" width="17.88671875" style="1" customWidth="1"/>
+    <col min="6" max="8" width="17.6640625" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="5" t="s">
         <v>6</v>
       </c>
+      <c r="G1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="3">
+    <row r="2" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="6">
         <v>44874</v>
       </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3">
+      <c r="D2" s="7"/>
+      <c r="E2" s="6">
         <v>44875</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" s="7"/>
     </row>
-    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="9" t="s">
         <v>10</v>
       </c>
+      <c r="E3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="8"/>
+      <c r="H3" s="9"/>
     </row>
-    <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="9" t="s">
         <v>9</v>
       </c>
+      <c r="E4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="8"/>
+      <c r="H4" s="9"/>
     </row>
-    <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="9" t="s">
         <v>9</v>
       </c>
+      <c r="E5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="8"/>
+      <c r="H5" s="9"/>
     </row>
-    <row r="6" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="9" t="s">
         <v>11</v>
       </c>
+      <c r="E6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="8"/>
+      <c r="H6" s="9"/>
     </row>
-    <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:8" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="11" t="s">
         <v>10</v>
       </c>
+      <c r="E7" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="10"/>
+      <c r="H7" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update schematic + docs
</commit_message>
<xml_diff>
--- a/MongoDB/Sprint reviews.xlsx
+++ b/MongoDB/Sprint reviews.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="101" documentId="13_ncr:1_{D4C4D4CE-E39E-4092-9DCE-47B9159D051B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E59420D2-7A23-48DD-9C8C-2E5F865BF363}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="330" windowWidth="29040" windowHeight="15990" xr2:uid="{40B4DD2A-A988-466C-98BC-3488A5760252}"/>
+    <workbookView minimized="1" xWindow="384" yWindow="840" windowWidth="17280" windowHeight="9072" xr2:uid="{40B4DD2A-A988-466C-98BC-3488A5760252}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint reviews" sheetId="1" r:id="rId1"/>
@@ -285,19 +285,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -316,10 +316,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -678,34 +674,34 @@
       </c>
     </row>
     <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="10">
+      <c r="B2" s="13">
         <v>44874</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="10">
+      <c r="C2" s="14"/>
+      <c r="D2" s="13">
         <v>44875</v>
       </c>
-      <c r="E2" s="11"/>
-      <c r="F2" s="10">
+      <c r="E2" s="14"/>
+      <c r="F2" s="13">
         <v>44876</v>
       </c>
-      <c r="G2" s="11"/>
-      <c r="H2" s="10">
+      <c r="G2" s="14"/>
+      <c r="H2" s="13">
         <v>44879</v>
       </c>
-      <c r="I2" s="11"/>
-      <c r="J2" s="10">
+      <c r="I2" s="14"/>
+      <c r="J2" s="13">
         <v>44881</v>
       </c>
-      <c r="K2" s="11"/>
-      <c r="L2" s="10">
+      <c r="K2" s="14"/>
+      <c r="L2" s="13">
         <v>44883</v>
       </c>
-      <c r="M2" s="11"/>
-      <c r="N2" s="10" t="s">
+      <c r="M2" s="14"/>
+      <c r="N2" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="O2" s="11"/>
+      <c r="O2" s="14"/>
     </row>
     <row r="3" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -730,11 +726,11 @@
         <v>10</v>
       </c>
       <c r="H3" s="6"/>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="12" t="s">
         <v>28</v>
       </c>
       <c r="J3" s="6"/>
-      <c r="K3" s="13" t="s">
+      <c r="K3" s="12" t="s">
         <v>30</v>
       </c>
       <c r="L3" s="6"/>
@@ -765,9 +761,9 @@
         <v>16</v>
       </c>
       <c r="H4" s="6"/>
-      <c r="I4" s="13"/>
+      <c r="I4" s="12"/>
       <c r="J4" s="6"/>
-      <c r="K4" s="13"/>
+      <c r="K4" s="12"/>
       <c r="L4" s="6"/>
       <c r="M4" s="7"/>
       <c r="N4" s="6"/>
@@ -796,9 +792,9 @@
         <v>15</v>
       </c>
       <c r="H5" s="6"/>
-      <c r="I5" s="13"/>
+      <c r="I5" s="12"/>
       <c r="J5" s="6"/>
-      <c r="K5" s="13"/>
+      <c r="K5" s="12"/>
       <c r="L5" s="6"/>
       <c r="M5" s="7"/>
       <c r="N5" s="6"/>
@@ -875,59 +871,59 @@
       <c r="O7" s="9"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H9" s="12" t="s">
+      <c r="H9" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12" t="s">
+      <c r="I9" s="10"/>
+      <c r="J9" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12" t="s">
+      <c r="K9" s="10"/>
+      <c r="L9" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12" t="s">
+      <c r="M9" s="10"/>
+      <c r="N9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="O9" s="12"/>
+      <c r="O9" s="10"/>
     </row>
     <row r="12" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="H12" s="12" t="s">
+      <c r="H12" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="I12" s="12"/>
+      <c r="I12" s="10"/>
       <c r="L12" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H15" s="14" t="s">
+      <c r="H15" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="I15" s="14"/>
+      <c r="I15" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="K3:K5"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N2:O2"/>
     <mergeCell ref="N9:O9"/>
     <mergeCell ref="H15:I15"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="H12:I13"/>
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="K3:K5"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
MongoDB.docx & SprintReview.xlsx updates
</commit_message>
<xml_diff>
--- a/MongoDB/Sprint reviews.xlsx
+++ b/MongoDB/Sprint reviews.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10661916_polimi_it/Documents/PoliMi/4° anno/Corsi/Systems and Methods for Big and Unstructured Data/Project SMBUD/SMBUD DB/Repository/SMBUD-project2022/MongoDB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="13_ncr:1_{D4C4D4CE-E39E-4092-9DCE-47B9159D051B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E59420D2-7A23-48DD-9C8C-2E5F865BF363}"/>
+  <xr:revisionPtr revIDLastSave="121" documentId="13_ncr:1_{D4C4D4CE-E39E-4092-9DCE-47B9159D051B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAA55527-31C7-4BFB-8A29-262EACE07F8D}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="384" yWindow="840" windowWidth="17280" windowHeight="9072" xr2:uid="{40B4DD2A-A988-466C-98BC-3488A5760252}"/>
+    <workbookView xWindow="-28920" yWindow="330" windowWidth="29040" windowHeight="15990" xr2:uid="{40B4DD2A-A988-466C-98BC-3488A5760252}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint reviews" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="39">
   <si>
     <t>Francesco</t>
   </si>
@@ -128,16 +128,31 @@
     <t>script python modules + Importing data in DB (w/Marco) + generated JSON with ref from py ready to import in DB</t>
   </si>
   <si>
-    <t>Latex w/ previous queries ready + 1q+2comm</t>
-  </si>
-  <si>
     <t>Revision</t>
   </si>
   <si>
-    <t>To check complexity of queries</t>
-  </si>
-  <si>
     <t>Latex ready</t>
+  </si>
+  <si>
+    <t>3q + 1c</t>
+  </si>
+  <si>
+    <t>2q + 2q (riserva)</t>
+  </si>
+  <si>
+    <t>1q + 2c + latex intro part</t>
+  </si>
+  <si>
+    <t>Latex w/ previous queries  + 2q+1comm + cambiare lo schema per array immagini (rimuovere) + cambiare nome da section a section array</t>
+  </si>
+  <si>
+    <t>check correctness latex (+comments)</t>
+  </si>
+  <si>
+    <t>To check complexity of queries -&gt; OK</t>
+  </si>
+  <si>
+    <t>18-19/11/2022</t>
   </si>
 </sst>
 </file>
@@ -162,7 +177,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -177,7 +192,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -256,7 +271,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -285,24 +300,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Accent4" xfId="1" builtinId="41"/>
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -674,34 +692,34 @@
       </c>
     </row>
     <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="13">
+      <c r="B2" s="10">
         <v>44874</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="13">
+      <c r="C2" s="11"/>
+      <c r="D2" s="10">
         <v>44875</v>
       </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="13">
+      <c r="E2" s="11"/>
+      <c r="F2" s="10">
         <v>44876</v>
       </c>
-      <c r="G2" s="14"/>
-      <c r="H2" s="13">
+      <c r="G2" s="11"/>
+      <c r="H2" s="10">
         <v>44879</v>
       </c>
-      <c r="I2" s="14"/>
-      <c r="J2" s="13">
+      <c r="I2" s="11"/>
+      <c r="J2" s="10">
         <v>44881</v>
       </c>
-      <c r="K2" s="14"/>
-      <c r="L2" s="13">
-        <v>44883</v>
-      </c>
-      <c r="M2" s="14"/>
-      <c r="N2" s="13" t="s">
+      <c r="K2" s="11"/>
+      <c r="L2" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="M2" s="11"/>
+      <c r="N2" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="O2" s="14"/>
+      <c r="O2" s="11"/>
     </row>
     <row r="3" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -725,16 +743,20 @@
       <c r="G3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="6"/>
+      <c r="H3" s="14" t="s">
+        <v>34</v>
+      </c>
       <c r="I3" s="12" t="s">
         <v>28</v>
       </c>
       <c r="J3" s="6"/>
       <c r="K3" s="12" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="L3" s="6"/>
-      <c r="M3" s="7"/>
+      <c r="M3" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="N3" s="6"/>
       <c r="O3" s="7"/>
     </row>
@@ -760,12 +782,12 @@
       <c r="G4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="6"/>
+      <c r="H4" s="14"/>
       <c r="I4" s="12"/>
       <c r="J4" s="6"/>
       <c r="K4" s="12"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="7"/>
+      <c r="M4" s="12"/>
       <c r="N4" s="6"/>
       <c r="O4" s="7"/>
     </row>
@@ -791,12 +813,12 @@
       <c r="G5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="6"/>
+      <c r="H5" s="14"/>
       <c r="I5" s="12"/>
       <c r="J5" s="6"/>
       <c r="K5" s="12"/>
       <c r="L5" s="6"/>
-      <c r="M5" s="7"/>
+      <c r="M5" s="12"/>
       <c r="N5" s="6"/>
       <c r="O5" s="7"/>
     </row>
@@ -822,7 +844,9 @@
       <c r="G6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="6"/>
+      <c r="H6" s="6" t="s">
+        <v>33</v>
+      </c>
       <c r="I6" s="7" t="s">
         <v>21</v>
       </c>
@@ -831,7 +855,9 @@
         <v>26</v>
       </c>
       <c r="L6" s="6"/>
-      <c r="M6" s="7"/>
+      <c r="M6" s="7" t="s">
+        <v>36</v>
+      </c>
       <c r="N6" s="6"/>
       <c r="O6" s="7"/>
     </row>
@@ -857,7 +883,9 @@
       <c r="G7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="8"/>
+      <c r="H7" s="8" t="s">
+        <v>32</v>
+      </c>
       <c r="I7" s="9" t="s">
         <v>20</v>
       </c>
@@ -866,64 +894,68 @@
         <v>27</v>
       </c>
       <c r="L7" s="8"/>
-      <c r="M7" s="9"/>
+      <c r="M7" s="9" t="s">
+        <v>36</v>
+      </c>
       <c r="N7" s="8"/>
       <c r="O7" s="9"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10" t="s">
+      <c r="I9" s="13"/>
+      <c r="J9" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10" t="s">
+      <c r="K9" s="13"/>
+      <c r="L9" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="O9" s="10"/>
+      <c r="M9" s="13"/>
+      <c r="N9" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="O9" s="13"/>
     </row>
     <row r="12" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="I12" s="10"/>
+      <c r="I12" s="13"/>
       <c r="L12" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H15" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="I15" s="11"/>
+      <c r="H15" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="I15" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="17">
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H12:I13"/>
+    <mergeCell ref="K3:K5"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="M3:M5"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="I3:I5"/>
-    <mergeCell ref="K3:K5"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H12:I13"/>
+    <mergeCell ref="H3:H5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
17/11 Sprint review updates
</commit_message>
<xml_diff>
--- a/MongoDB/Sprint reviews.xlsx
+++ b/MongoDB/Sprint reviews.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10661916_polimi_it/Documents/PoliMi/4° anno/Corsi/Systems and Methods for Big and Unstructured Data/Project SMBUD/SMBUD DB/Repository/SMBUD-project2022/MongoDB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="121" documentId="13_ncr:1_{D4C4D4CE-E39E-4092-9DCE-47B9159D051B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAA55527-31C7-4BFB-8A29-262EACE07F8D}"/>
+  <xr:revisionPtr revIDLastSave="128" documentId="13_ncr:1_{D4C4D4CE-E39E-4092-9DCE-47B9159D051B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F60A3BD9-4624-41F6-A689-224BB811FBCF}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="330" windowWidth="29040" windowHeight="15990" xr2:uid="{40B4DD2A-A988-466C-98BC-3488A5760252}"/>
+    <workbookView xWindow="-108" yWindow="348" windowWidth="23256" windowHeight="12720" xr2:uid="{40B4DD2A-A988-466C-98BC-3488A5760252}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint reviews" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,72 +36,102 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="42">
+  <si>
+    <t>What done</t>
+  </si>
+  <si>
+    <t>Expected</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
   <si>
     <t>Francesco</t>
   </si>
   <si>
+    <t>Analysis</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Learning about importing in MongoDB</t>
+  </si>
+  <si>
+    <t>check progress and correctness schema + Importing data in DB (w/Marco)</t>
+  </si>
+  <si>
+    <t>1q + 2c + latex intro part</t>
+  </si>
+  <si>
+    <t>Latex intro part + importing + 2q+1comm</t>
+  </si>
+  <si>
+    <t>Latex w/ previous queries  + 2q+1comm + cambiare lo schema per array immagini (rimuovere) + cambiare nome da sections a section array</t>
+  </si>
+  <si>
+    <t>Latex ready</t>
+  </si>
+  <si>
     <t>Alessandro</t>
   </si>
   <si>
+    <t>Analysis, document schema</t>
+  </si>
+  <si>
+    <t>Random data generation process</t>
+  </si>
+  <si>
+    <t>Learning Json py lib</t>
+  </si>
+  <si>
+    <t>py from txt to json for book text</t>
+  </si>
+  <si>
     <t>Marco</t>
   </si>
   <si>
+    <t>script python modules + Importing data in DB (w/Marco) + generated JSON with ref from py ready to import in DB</t>
+  </si>
+  <si>
+    <t>progress in random data generation</t>
+  </si>
+  <si>
     <t>Lorenzo</t>
   </si>
   <si>
+    <t>document schema</t>
+  </si>
+  <si>
+    <t>Check correctness document schema</t>
+  </si>
+  <si>
+    <t>2q + 2q (riserva)</t>
+  </si>
+  <si>
+    <t>Check correctness document schema + 3q + 1 command</t>
+  </si>
+  <si>
+    <t>2q +1c</t>
+  </si>
+  <si>
+    <t>check correctness latex (+comments)</t>
+  </si>
+  <si>
     <t>Simone</t>
   </si>
   <si>
-    <t>What done</t>
-  </si>
-  <si>
-    <t>Expected</t>
-  </si>
-  <si>
-    <t>Analysis</t>
-  </si>
-  <si>
-    <t>document schema</t>
-  </si>
-  <si>
-    <t>Learning Json py lib</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Check correctness document schema</t>
-  </si>
-  <si>
-    <t>Analysis, document schema</t>
-  </si>
-  <si>
     <t>Latex template</t>
   </si>
   <si>
-    <t>Random data generation process</t>
-  </si>
-  <si>
-    <t>progress in random data generation</t>
-  </si>
-  <si>
-    <t>py from txt to json for book text</t>
-  </si>
-  <si>
-    <t>Learning about importing in MongoDB</t>
-  </si>
-  <si>
-    <t>?</t>
-  </si>
-  <si>
-    <t>check progress and correctness schema + Importing data in DB (w/Marco)</t>
+    <t>3q + 1c</t>
   </si>
   <si>
     <t>3q + 1 command</t>
   </si>
   <si>
-    <t>Check correctness document schema + 3q + 1 command</t>
+    <t>2q+1c</t>
   </si>
   <si>
     <t>Needed: 50% queries ready</t>
@@ -110,49 +140,28 @@
     <t>Needed: Queries ready</t>
   </si>
   <si>
+    <t>Revision</t>
+  </si>
+  <si>
     <t>Each query on mongodb doc queries with desc. In english (so they are better described)</t>
   </si>
   <si>
     <t>Needed: 10q + 5 comm, we do 13q+7 comm</t>
   </si>
   <si>
-    <t>2q +1c</t>
-  </si>
-  <si>
-    <t>2q+1c</t>
-  </si>
-  <si>
-    <t>Latex intro part + importing + 2q+1comm</t>
-  </si>
-  <si>
-    <t>script python modules + Importing data in DB (w/Marco) + generated JSON with ref from py ready to import in DB</t>
-  </si>
-  <si>
-    <t>Revision</t>
-  </si>
-  <si>
-    <t>Latex ready</t>
-  </si>
-  <si>
-    <t>3q + 1c</t>
-  </si>
-  <si>
-    <t>2q + 2q (riserva)</t>
-  </si>
-  <si>
-    <t>1q + 2c + latex intro part</t>
-  </si>
-  <si>
-    <t>Latex w/ previous queries  + 2q+1comm + cambiare lo schema per array immagini (rimuovere) + cambiare nome da section a section array</t>
-  </si>
-  <si>
-    <t>check correctness latex (+comments)</t>
-  </si>
-  <si>
     <t>To check complexity of queries -&gt; OK</t>
   </si>
   <si>
-    <t>18-19/11/2022</t>
+    <t>Array images removed + decided not to change the name section/section array</t>
+  </si>
+  <si>
+    <t>2q + 1c</t>
+  </si>
+  <si>
+    <t>20/11/2022 - 21.00</t>
+  </si>
+  <si>
+    <t>???</t>
   </si>
 </sst>
 </file>
@@ -309,10 +318,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
@@ -643,52 +652,52 @@
     <col min="7" max="7" width="17.6640625" style="1" customWidth="1"/>
     <col min="8" max="10" width="23.44140625" style="1" customWidth="1"/>
     <col min="11" max="12" width="23.109375" style="1" customWidth="1"/>
-    <col min="13" max="15" width="22.77734375" style="1" customWidth="1"/>
+    <col min="13" max="15" width="22.6640625" style="1" customWidth="1"/>
     <col min="16" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B1" s="4" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -713,68 +722,70 @@
       </c>
       <c r="K2" s="11"/>
       <c r="L2" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="M2" s="11"/>
       <c r="N2" s="10" t="s">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="O2" s="11"/>
     </row>
     <row r="3" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="G3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="K3" s="12" t="s">
         <v>10</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" s="6"/>
-      <c r="K3" s="12" t="s">
-        <v>35</v>
       </c>
       <c r="L3" s="6"/>
       <c r="M3" s="12" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="N3" s="6"/>
       <c r="O3" s="7"/>
     </row>
     <row r="4" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>16</v>
@@ -782,9 +793,9 @@
       <c r="G4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="14"/>
+      <c r="H4" s="13"/>
       <c r="I4" s="12"/>
-      <c r="J4" s="6"/>
+      <c r="J4" s="13"/>
       <c r="K4" s="12"/>
       <c r="L4" s="6"/>
       <c r="M4" s="12"/>
@@ -793,29 +804,29 @@
     </row>
     <row r="5" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" s="14"/>
+        <v>19</v>
+      </c>
+      <c r="H5" s="13"/>
       <c r="I5" s="12"/>
-      <c r="J5" s="6"/>
+      <c r="J5" s="13"/>
       <c r="K5" s="12"/>
       <c r="L5" s="6"/>
       <c r="M5" s="12"/>
@@ -824,112 +835,116 @@
     </row>
     <row r="6" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J6" s="6"/>
+        <v>24</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>41</v>
+      </c>
       <c r="K6" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L6" s="6"/>
       <c r="M6" s="7" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="N6" s="6"/>
       <c r="O6" s="7"/>
     </row>
     <row r="7" spans="1:15" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" s="8"/>
+        <v>30</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>39</v>
+      </c>
       <c r="K7" s="9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="L7" s="8"/>
       <c r="M7" s="9" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="N7" s="8"/>
       <c r="O7" s="9"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H9" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="M9" s="13"/>
-      <c r="N9" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="O9" s="13"/>
+      <c r="H9" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K9" s="14"/>
+      <c r="L9" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="M9" s="14"/>
+      <c r="N9" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="O9" s="14"/>
     </row>
     <row r="12" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="H12" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="I12" s="13"/>
+      <c r="H12" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="I12" s="14"/>
       <c r="L12" s="1" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="H15" s="15" t="s">
@@ -938,7 +953,7 @@
       <c r="I15" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="H15:I15"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="J9:K9"/>
@@ -950,6 +965,7 @@
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="N9:O9"/>
     <mergeCell ref="M3:M5"/>
+    <mergeCell ref="J3:J5"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F2:G2"/>

</xml_diff>

<commit_message>
Updates ER, Queries.docx and SprintReviev.xlsx
</commit_message>
<xml_diff>
--- a/MongoDB/Sprint reviews.xlsx
+++ b/MongoDB/Sprint reviews.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10661916_polimi_it/Documents/PoliMi/4° anno/Corsi/Systems and Methods for Big and Unstructured Data/Project SMBUD/SMBUD DB/Repository/SMBUD-project2022/MongoDB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="222" documentId="13_ncr:1_{D4C4D4CE-E39E-4092-9DCE-47B9159D051B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99F13083-8B3D-4FB2-803A-354CE7097AD6}"/>
+  <xr:revisionPtr revIDLastSave="234" documentId="13_ncr:1_{D4C4D4CE-E39E-4092-9DCE-47B9159D051B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B99B4C5-DAA7-46A7-A599-552CE079B2F0}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="330" windowWidth="29040" windowHeight="15990" xr2:uid="{40B4DD2A-A988-466C-98BC-3488A5760252}"/>
+    <workbookView xWindow="-108" yWindow="348" windowWidth="23256" windowHeight="12720" xr2:uid="{40B4DD2A-A988-466C-98BC-3488A5760252}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint reviews" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="51">
   <si>
     <t>What done</t>
   </si>
@@ -164,9 +164,6 @@
     <t>Complexity, correctness of the queries</t>
   </si>
   <si>
-    <t>Revision Neo4J - 2 - 3 - 4 - c4 - c3 - c2</t>
-  </si>
-  <si>
     <t>Check correctness mongo db + revision 14 -15 - 9 - c1 - c7 - 8</t>
   </si>
   <si>
@@ -186,6 +183,12 @@
   </si>
   <si>
     <t>Things ready for delivery</t>
+  </si>
+  <si>
+    <t>Revision Neo4J (ER) - 2 - 3 - 4 - c4 - c3 - c2</t>
+  </si>
+  <si>
+    <t>Revision Neo4J + finish import mongo db description</t>
   </si>
 </sst>
 </file>
@@ -335,7 +338,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -367,47 +370,41 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -426,10 +423,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -777,7 +770,7 @@
       <c r="L1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="M1" s="19" t="s">
+      <c r="M1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="N1" s="4" t="s">
@@ -788,34 +781,34 @@
       </c>
     </row>
     <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="11">
+      <c r="B2" s="19">
         <v>44874</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="11">
+      <c r="C2" s="20"/>
+      <c r="D2" s="19">
         <v>44875</v>
       </c>
-      <c r="E2" s="12"/>
-      <c r="F2" s="11">
+      <c r="E2" s="20"/>
+      <c r="F2" s="19">
         <v>44876</v>
       </c>
-      <c r="G2" s="12"/>
-      <c r="H2" s="11">
+      <c r="G2" s="20"/>
+      <c r="H2" s="19">
         <v>44879</v>
       </c>
-      <c r="I2" s="12"/>
-      <c r="J2" s="11">
+      <c r="I2" s="20"/>
+      <c r="J2" s="19">
         <v>44882</v>
       </c>
-      <c r="K2" s="12"/>
-      <c r="L2" s="11" t="s">
+      <c r="K2" s="20"/>
+      <c r="L2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="20"/>
-      <c r="N2" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="O2" s="12"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="O2" s="20"/>
     </row>
     <row r="3" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -839,27 +832,29 @@
       <c r="G3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="H3" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="14" t="s">
+      <c r="J3" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="13" t="s">
+      <c r="K3" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="14" t="s">
+      <c r="L3" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="M3" s="21" t="s">
+      <c r="M3" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="N3" s="18"/>
-      <c r="O3" s="24" t="s">
-        <v>46</v>
+      <c r="N3" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="O3" s="14" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.3">
@@ -884,15 +879,17 @@
       <c r="G4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="14"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="18"/>
-      <c r="O4" s="24" t="s">
-        <v>45</v>
+      <c r="H4" s="22"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.3">
@@ -917,15 +914,17 @@
       <c r="G5" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="14"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="21"/>
-      <c r="N5" s="6"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="6" t="s">
+        <v>50</v>
+      </c>
       <c r="O5" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.3">
@@ -965,12 +964,14 @@
       <c r="L6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="M6" s="22" t="s">
+      <c r="M6" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="N6" s="6"/>
+      <c r="N6" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="O6" s="7" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1010,12 +1011,14 @@
       <c r="L7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="M7" s="23" t="s">
+      <c r="M7" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="N7" s="8"/>
+      <c r="N7" s="8" t="s">
+        <v>42</v>
+      </c>
       <c r="O7" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -1031,22 +1034,22 @@
         <v>12</v>
       </c>
       <c r="M9" s="16"/>
-      <c r="N9" s="15" t="s">
+      <c r="N9" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="O9" s="15"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="N10" s="15" t="s">
+      <c r="O9" s="16"/>
+    </row>
+    <row r="10" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N10" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="O10" s="15"/>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="N11" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="O11" s="15"/>
+      <c r="O10" s="16"/>
+    </row>
+    <row r="11" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N11" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="O11" s="17"/>
     </row>
     <row r="12" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="H12" s="16" t="s">
@@ -1056,10 +1059,10 @@
       <c r="L12" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="N12" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="O12" s="15"/>
+      <c r="N12" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="O12" s="16"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="H13" s="16"/>
@@ -1073,6 +1076,20 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="K3:K5"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="M3:M5"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="L3:L5"/>
     <mergeCell ref="N10:O10"/>
     <mergeCell ref="N11:O11"/>
     <mergeCell ref="N12:O12"/>
@@ -1081,20 +1098,6 @@
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="H12:I13"/>
-    <mergeCell ref="K3:K5"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="M3:M5"/>
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="L3:L5"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="H3:H5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>